<commit_message>
Ass exercise 4 to 8
</commit_message>
<xml_diff>
--- a/Advexcel/(Ass)Create from selection and Dates - Stu.xlsx(Date Function).xlsx
+++ b/Advexcel/(Ass)Create from selection and Dates - Stu.xlsx(Date Function).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/karan/Desktop/EXCEL ITVEDANT/Advexcel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28CE47E3-8B33-D849-8952-05C9E0D1E5F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88FFDEE5-7296-BE4B-9A00-B5897A6BE818}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Create from selection" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="259">
   <si>
     <t>Month</t>
   </si>
@@ -756,6 +756,72 @@
   </si>
   <si>
     <t>Last day of Completion month</t>
+  </si>
+  <si>
+    <t>Maturity Date</t>
+  </si>
+  <si>
+    <t>Maturity Year</t>
+  </si>
+  <si>
+    <t>Maturity Month</t>
+  </si>
+  <si>
+    <t>Last day of maturity month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Due Day Name </t>
+  </si>
+  <si>
+    <t>Due Month</t>
+  </si>
+  <si>
+    <t>Last day of due month</t>
+  </si>
+  <si>
+    <t>Weekday</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Month Name </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Week Number </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Days remaining until the event </t>
+  </si>
+  <si>
+    <t>last day of the event month</t>
+  </si>
+  <si>
+    <t>Current Age</t>
+  </si>
+  <si>
+    <t>Years of Experience</t>
+  </si>
+  <si>
+    <t>Joining Weekday</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Joining month name </t>
+  </si>
+  <si>
+    <t>Project duration in days</t>
+  </si>
+  <si>
+    <t>Project working days</t>
+  </si>
+  <si>
+    <t>Project completion month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 Months to the joining date </t>
+  </si>
+  <si>
+    <t>1 yeat the project lasted</t>
+  </si>
+  <si>
+    <t>last day pf project completion month</t>
   </si>
 </sst>
 </file>
@@ -833,7 +899,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -856,22 +922,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -944,18 +999,20 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1363,28 +1420,32 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39115F3F-0BAE-4E23-88D3-307E83662290}">
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:O23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.33203125" customWidth="1"/>
     <col min="2" max="2" width="9.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="20.1640625" customWidth="1"/>
-    <col min="11" max="11" width="17" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.83203125" customWidth="1"/>
+    <col min="8" max="8" width="9.6640625" customWidth="1"/>
+    <col min="10" max="10" width="14" customWidth="1"/>
+    <col min="11" max="11" width="12.33203125" customWidth="1"/>
+    <col min="12" max="13" width="9.6640625" customWidth="1"/>
+    <col min="14" max="14" width="9.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="31" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:15" ht="31" x14ac:dyDescent="0.2">
       <c r="A1" s="13" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="24" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:15" ht="24" x14ac:dyDescent="0.2">
       <c r="A3" s="12" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="32" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:15" ht="64" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>11</v>
       </c>
@@ -1400,8 +1461,38 @@
       <c r="E5" s="3" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F5" s="32" t="s">
+        <v>249</v>
+      </c>
+      <c r="G5" s="32" t="s">
+        <v>250</v>
+      </c>
+      <c r="H5" s="32" t="s">
+        <v>251</v>
+      </c>
+      <c r="I5" s="32" t="s">
+        <v>252</v>
+      </c>
+      <c r="J5" s="32" t="s">
+        <v>253</v>
+      </c>
+      <c r="K5" s="32" t="s">
+        <v>254</v>
+      </c>
+      <c r="L5" s="32" t="s">
+        <v>255</v>
+      </c>
+      <c r="M5" s="32" t="s">
+        <v>258</v>
+      </c>
+      <c r="N5" s="32" t="s">
+        <v>256</v>
+      </c>
+      <c r="O5" s="32" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>18</v>
       </c>
@@ -1417,8 +1508,48 @@
       <c r="E6" s="7">
         <v>46280</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F6" s="26">
+        <f ca="1">DATEDIF(C6,TODAY(),"y")</f>
+        <v>28</v>
+      </c>
+      <c r="G6" s="26">
+        <f ca="1">DATEDIF(B6,TODAY(),"y")</f>
+        <v>6</v>
+      </c>
+      <c r="H6" s="26" t="str">
+        <f>TEXT(B6,"dddd")</f>
+        <v>Wednesday</v>
+      </c>
+      <c r="I6" s="26" t="str">
+        <f>TEXT(B6,"mmmm")</f>
+        <v>January</v>
+      </c>
+      <c r="J6" s="37">
+        <f>D6-E6</f>
+        <v>-67</v>
+      </c>
+      <c r="K6" s="26">
+        <f>NETWORKDAYS(D6,E6)</f>
+        <v>48</v>
+      </c>
+      <c r="L6" s="26" t="str">
+        <f>TEXT(E6,"mmmm")</f>
+        <v>September</v>
+      </c>
+      <c r="M6" s="27">
+        <f>EOMONTH(E6,0)</f>
+        <v>46295</v>
+      </c>
+      <c r="N6" s="27">
+        <f>EDATE(B6,3)</f>
+        <v>43936</v>
+      </c>
+      <c r="O6" s="33">
+        <f>YEARFRAC(D6,E6)</f>
+        <v>0.18055555555555555</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -1434,8 +1565,48 @@
       <c r="E7" s="7">
         <v>46323</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F7" s="26">
+        <f t="shared" ref="F7:F10" ca="1" si="0">DATEDIF(C7,TODAY(),"y")</f>
+        <v>26</v>
+      </c>
+      <c r="G7" s="26">
+        <f t="shared" ref="G7:G10" ca="1" si="1">DATEDIF(B7,TODAY(),"y")</f>
+        <v>5</v>
+      </c>
+      <c r="H7" s="26" t="str">
+        <f t="shared" ref="H7:H10" si="2">TEXT(B7,"dddd")</f>
+        <v>Thursday</v>
+      </c>
+      <c r="I7" s="26" t="str">
+        <f t="shared" ref="I7:I10" si="3">TEXT(B7,"mmmm")</f>
+        <v>March</v>
+      </c>
+      <c r="J7" s="26">
+        <f t="shared" ref="J7:J10" si="4">D7-E7</f>
+        <v>-105</v>
+      </c>
+      <c r="K7" s="26">
+        <f t="shared" ref="K7:K10" si="5">NETWORKDAYS(D7,E7)</f>
+        <v>76</v>
+      </c>
+      <c r="L7" s="26" t="str">
+        <f t="shared" ref="L7:L10" si="6">TEXT(E7,"mmmm")</f>
+        <v>October</v>
+      </c>
+      <c r="M7" s="27">
+        <f t="shared" ref="M7:M10" si="7">EOMONTH(E7,0)</f>
+        <v>46326</v>
+      </c>
+      <c r="N7" s="27">
+        <f t="shared" ref="N7:N10" si="8">EDATE(B7,3)</f>
+        <v>44365</v>
+      </c>
+      <c r="O7" s="33">
+        <f t="shared" ref="O7:O10" si="9">YEARFRAC(D7,E7)</f>
+        <v>0.28611111111111109</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>22</v>
       </c>
@@ -1451,8 +1622,48 @@
       <c r="E8" s="7">
         <v>46368</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F8" s="26">
+        <f t="shared" ca="1" si="0"/>
+        <v>28</v>
+      </c>
+      <c r="G8" s="26">
+        <f t="shared" ca="1" si="1"/>
+        <v>7</v>
+      </c>
+      <c r="H8" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v>Tuesday</v>
+      </c>
+      <c r="I8" s="26" t="str">
+        <f t="shared" si="3"/>
+        <v>June</v>
+      </c>
+      <c r="J8" s="26">
+        <f t="shared" si="4"/>
+        <v>-145</v>
+      </c>
+      <c r="K8" s="26">
+        <f t="shared" si="5"/>
+        <v>105</v>
+      </c>
+      <c r="L8" s="26" t="str">
+        <f t="shared" si="6"/>
+        <v>December</v>
+      </c>
+      <c r="M8" s="27">
+        <f t="shared" si="7"/>
+        <v>46387</v>
+      </c>
+      <c r="N8" s="27">
+        <f t="shared" si="8"/>
+        <v>43733</v>
+      </c>
+      <c r="O8" s="33">
+        <f t="shared" si="9"/>
+        <v>0.39444444444444443</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>24</v>
       </c>
@@ -1468,8 +1679,48 @@
       <c r="E9" s="7">
         <v>46344</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F9" s="26">
+        <f t="shared" ca="1" si="0"/>
+        <v>30</v>
+      </c>
+      <c r="G9" s="26">
+        <f t="shared" ca="1" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="H9" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v>Saturday</v>
+      </c>
+      <c r="I9" s="26" t="str">
+        <f t="shared" si="3"/>
+        <v>February</v>
+      </c>
+      <c r="J9" s="26">
+        <f t="shared" si="4"/>
+        <v>-116</v>
+      </c>
+      <c r="K9" s="26">
+        <f t="shared" si="5"/>
+        <v>83</v>
+      </c>
+      <c r="L9" s="26" t="str">
+        <f t="shared" si="6"/>
+        <v>November</v>
+      </c>
+      <c r="M9" s="27">
+        <f t="shared" si="7"/>
+        <v>46356</v>
+      </c>
+      <c r="N9" s="27">
+        <f t="shared" si="8"/>
+        <v>44693</v>
+      </c>
+      <c r="O9" s="33">
+        <f t="shared" si="9"/>
+        <v>0.31388888888888888</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>26</v>
       </c>
@@ -1485,26 +1736,66 @@
       <c r="E10" s="7">
         <v>46409</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" ht="19" x14ac:dyDescent="0.2">
+      <c r="F10" s="26">
+        <f t="shared" ca="1" si="0"/>
+        <v>31</v>
+      </c>
+      <c r="G10" s="26">
+        <f t="shared" ca="1" si="1"/>
+        <v>8</v>
+      </c>
+      <c r="H10" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v>Wednesday</v>
+      </c>
+      <c r="I10" s="26" t="str">
+        <f t="shared" si="3"/>
+        <v>August</v>
+      </c>
+      <c r="J10" s="26">
+        <f t="shared" si="4"/>
+        <v>-176</v>
+      </c>
+      <c r="K10" s="26">
+        <f t="shared" si="5"/>
+        <v>127</v>
+      </c>
+      <c r="L10" s="26" t="str">
+        <f t="shared" si="6"/>
+        <v>January</v>
+      </c>
+      <c r="M10" s="27">
+        <f t="shared" si="7"/>
+        <v>46418</v>
+      </c>
+      <c r="N10" s="27">
+        <f t="shared" si="8"/>
+        <v>43412</v>
+      </c>
+      <c r="O10" s="33">
+        <f t="shared" si="9"/>
+        <v>0.4777777777777778</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" ht="19" x14ac:dyDescent="0.2">
       <c r="A12" s="14" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13" s="15"/>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A15" s="15" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A16" s="15" t="s">
         <v>194</v>
       </c>
@@ -1593,11 +1884,11 @@
       <c r="H1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="J1" s="29" t="s">
+      <c r="J1" s="31" t="s">
         <v>66</v>
       </c>
-      <c r="K1" s="29"/>
-      <c r="L1" s="29"/>
+      <c r="K1" s="31"/>
+      <c r="L1" s="31"/>
     </row>
     <row r="2" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="2">
@@ -1647,7 +1938,7 @@
       </c>
       <c r="G3" s="9">
         <f ca="1">NOW()</f>
-        <v>46297.026281597224</v>
+        <v>46297.7256494213</v>
       </c>
       <c r="H3" s="10">
         <v>46227.947916666664</v>
@@ -1733,7 +2024,7 @@
       </c>
       <c r="L5" s="9">
         <f ca="1">NOW()</f>
-        <v>46297.026281597224</v>
+        <v>46297.7256494213</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="17" x14ac:dyDescent="0.2">
@@ -2741,7 +3032,7 @@
       <c r="A15" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="D15" s="30"/>
+      <c r="D15" s="28"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" s="15" t="s">
@@ -2833,6 +3124,7 @@
   <cols>
     <col min="4" max="4" width="12.5" customWidth="1"/>
     <col min="6" max="6" width="11.5" customWidth="1"/>
+    <col min="7" max="7" width="10" customWidth="1"/>
     <col min="9" max="9" width="11.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2856,16 +3148,16 @@
       <c r="C5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="28" t="s">
+      <c r="D5" s="3" t="s">
         <v>225</v>
       </c>
-      <c r="E5" s="28" t="s">
+      <c r="E5" s="3" t="s">
         <v>224</v>
       </c>
-      <c r="F5" s="28" t="s">
+      <c r="F5" s="3" t="s">
         <v>226</v>
       </c>
-      <c r="G5" s="28" t="s">
+      <c r="G5" s="3" t="s">
         <v>227</v>
       </c>
     </row>
@@ -2879,19 +3171,19 @@
       <c r="C6" s="7">
         <v>46224</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="26">
         <f>C6-B6</f>
         <v>6</v>
       </c>
-      <c r="E6">
+      <c r="E6" s="26">
         <f>NETWORKDAYS(B6,C6)</f>
         <v>5</v>
       </c>
-      <c r="F6" s="18">
+      <c r="F6" s="27">
         <f>EOMONTH(C6,0)</f>
         <v>46234</v>
       </c>
-      <c r="G6" t="str">
+      <c r="G6" s="26" t="str">
         <f>TEXT(C6,"dddd")</f>
         <v>Tuesday</v>
       </c>
@@ -2906,19 +3198,19 @@
       <c r="C7" s="7">
         <v>46227</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="26">
         <f t="shared" ref="D7:D10" si="0">C7-B7</f>
         <v>8</v>
       </c>
-      <c r="E7">
+      <c r="E7" s="26">
         <f t="shared" ref="E7:E10" si="1">NETWORKDAYS(B7,C7)</f>
         <v>7</v>
       </c>
-      <c r="F7" s="18">
+      <c r="F7" s="27">
         <f t="shared" ref="F7:F10" si="2">EOMONTH(C7,0)</f>
         <v>46234</v>
       </c>
-      <c r="G7" t="str">
+      <c r="G7" s="26" t="str">
         <f t="shared" ref="G7:G10" si="3">TEXT(C7,"dddd")</f>
         <v>Friday</v>
       </c>
@@ -2933,19 +3225,19 @@
       <c r="C8" s="7">
         <v>46231</v>
       </c>
-      <c r="D8">
+      <c r="D8" s="26">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="E8">
+      <c r="E8" s="26">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
-      <c r="F8" s="18">
+      <c r="F8" s="27">
         <f t="shared" si="2"/>
         <v>46234</v>
       </c>
-      <c r="G8" t="str">
+      <c r="G8" s="26" t="str">
         <f t="shared" si="3"/>
         <v>Tuesday</v>
       </c>
@@ -2960,19 +3252,19 @@
       <c r="C9" s="7">
         <v>46228</v>
       </c>
-      <c r="D9">
+      <c r="D9" s="26">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="E9">
+      <c r="E9" s="26">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="F9" s="18">
+      <c r="F9" s="27">
         <f t="shared" si="2"/>
         <v>46234</v>
       </c>
-      <c r="G9" t="str">
+      <c r="G9" s="26" t="str">
         <f t="shared" si="3"/>
         <v>Saturday</v>
       </c>
@@ -2987,19 +3279,19 @@
       <c r="C10" s="7">
         <v>46232</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="26">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="E10">
+      <c r="E10" s="26">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="F10" s="18">
+      <c r="F10" s="27">
         <f t="shared" si="2"/>
         <v>46234</v>
       </c>
-      <c r="G10" t="str">
+      <c r="G10" s="26" t="str">
         <f t="shared" si="3"/>
         <v>Wednesday</v>
       </c>
@@ -3084,19 +3376,19 @@
       <c r="B5" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="C5" s="31" t="s">
+      <c r="C5" s="29" t="s">
         <v>228</v>
       </c>
-      <c r="D5" s="31" t="s">
+      <c r="D5" s="29" t="s">
         <v>229</v>
       </c>
-      <c r="E5" s="31" t="s">
+      <c r="E5" s="29" t="s">
         <v>230</v>
       </c>
-      <c r="F5" s="31" t="s">
+      <c r="F5" s="29" t="s">
         <v>232</v>
       </c>
-      <c r="G5" s="31" t="s">
+      <c r="G5" s="29" t="s">
         <v>231</v>
       </c>
     </row>
@@ -3111,7 +3403,7 @@
         <f ca="1">DATEDIF(B6,TODAY(),"y")</f>
         <v>22</v>
       </c>
-      <c r="D6" s="32" t="str">
+      <c r="D6" s="30" t="str">
         <f>TEXT(B6,"mm")</f>
         <v>03</v>
       </c>
@@ -3139,7 +3431,7 @@
         <f t="shared" ref="C7:C10" ca="1" si="0">DATEDIF(B7,TODAY(),"y")</f>
         <v>21</v>
       </c>
-      <c r="D7" s="32" t="str">
+      <c r="D7" s="30" t="str">
         <f t="shared" ref="D7:D10" si="1">TEXT(B7,"mm")</f>
         <v>01</v>
       </c>
@@ -3167,7 +3459,7 @@
         <f t="shared" ca="1" si="0"/>
         <v>22</v>
       </c>
-      <c r="D8" s="32" t="str">
+      <c r="D8" s="30" t="str">
         <f t="shared" si="1"/>
         <v>11</v>
       </c>
@@ -3195,7 +3487,7 @@
         <f t="shared" ca="1" si="0"/>
         <v>22</v>
       </c>
-      <c r="D9" s="32" t="str">
+      <c r="D9" s="30" t="str">
         <f t="shared" si="1"/>
         <v>07</v>
       </c>
@@ -3223,7 +3515,7 @@
         <f t="shared" ca="1" si="0"/>
         <v>20</v>
       </c>
-      <c r="D10" s="32" t="str">
+      <c r="D10" s="30" t="str">
         <f t="shared" si="1"/>
         <v>05</v>
       </c>
@@ -3301,7 +3593,7 @@
       </c>
     </row>
     <row r="4" spans="1:8" ht="23" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="5" spans="1:8" ht="64" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>144</v>
       </c>
@@ -3311,16 +3603,16 @@
       <c r="C5" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="D5" s="33" t="s">
+      <c r="D5" s="3" t="s">
         <v>233</v>
       </c>
-      <c r="E5" s="33" t="s">
+      <c r="E5" s="3" t="s">
         <v>234</v>
       </c>
-      <c r="F5" s="33" t="s">
+      <c r="F5" s="3" t="s">
         <v>235</v>
       </c>
-      <c r="G5" s="33" t="s">
+      <c r="G5" s="3" t="s">
         <v>236</v>
       </c>
     </row>
@@ -3338,7 +3630,7 @@
         <f>WORKDAY(B6,+C6)</f>
         <v>46281</v>
       </c>
-      <c r="E6" s="32" t="str">
+      <c r="E6" s="30" t="str">
         <f>TEXT(D6,"mmmm")</f>
         <v>September</v>
       </c>
@@ -3366,7 +3658,7 @@
         <f t="shared" ref="D7:D10" si="0">WORKDAY(B7,+C7)</f>
         <v>46265</v>
       </c>
-      <c r="E7" s="32" t="str">
+      <c r="E7" s="30" t="str">
         <f t="shared" ref="E7:E10" si="1">TEXT(D7,"mmmm")</f>
         <v>August</v>
       </c>
@@ -3378,6 +3670,7 @@
         <f t="shared" ref="G7:G10" si="3">EOMONTH(B7,0)</f>
         <v>46234</v>
       </c>
+      <c r="H7" s="18"/>
     </row>
     <row r="8" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
@@ -3393,7 +3686,7 @@
         <f t="shared" si="0"/>
         <v>46311</v>
       </c>
-      <c r="E8" s="32" t="str">
+      <c r="E8" s="30" t="str">
         <f t="shared" si="1"/>
         <v>October</v>
       </c>
@@ -3405,6 +3698,7 @@
         <f t="shared" si="3"/>
         <v>46234</v>
       </c>
+      <c r="H8" s="18"/>
     </row>
     <row r="9" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
@@ -3420,7 +3714,7 @@
         <f t="shared" si="0"/>
         <v>46301</v>
       </c>
-      <c r="E9" s="32" t="str">
+      <c r="E9" s="30" t="str">
         <f t="shared" si="1"/>
         <v>October</v>
       </c>
@@ -3432,6 +3726,7 @@
         <f t="shared" si="3"/>
         <v>46234</v>
       </c>
+      <c r="H9" s="18"/>
     </row>
     <row r="10" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
@@ -3447,7 +3742,7 @@
         <f t="shared" si="0"/>
         <v>46268</v>
       </c>
-      <c r="E10" s="32" t="str">
+      <c r="E10" s="30" t="str">
         <f t="shared" si="1"/>
         <v>September</v>
       </c>
@@ -3459,6 +3754,7 @@
         <f t="shared" si="3"/>
         <v>46234</v>
       </c>
+      <c r="H10" s="18"/>
     </row>
     <row r="12" spans="1:8" ht="19" x14ac:dyDescent="0.2">
       <c r="A12" s="14" t="s">
@@ -3495,26 +3791,24 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59132BF8-75B1-4B7E-BB13-589F75BA747C}">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="9.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.6640625" customWidth="1"/>
+    <col min="1" max="7" width="9.33203125" customWidth="1"/>
     <col min="9" max="9" width="14.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="31" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" ht="31" x14ac:dyDescent="0.2">
       <c r="A1" s="13" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="24" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" ht="24" x14ac:dyDescent="0.2">
       <c r="A3" s="12" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="32" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" ht="64" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>157</v>
       </c>
@@ -3524,8 +3818,20 @@
       <c r="C5" s="3" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="D5" s="32" t="s">
+        <v>237</v>
+      </c>
+      <c r="E5" s="32" t="s">
+        <v>238</v>
+      </c>
+      <c r="F5" s="32" t="s">
+        <v>239</v>
+      </c>
+      <c r="G5" s="32" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>18</v>
       </c>
@@ -3535,8 +3841,24 @@
       <c r="C6" s="2">
         <v>24</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="D6" s="27">
+        <f>EDATE(B6,C6)</f>
+        <v>46034</v>
+      </c>
+      <c r="E6" s="26">
+        <f>YEAR(D6)</f>
+        <v>2026</v>
+      </c>
+      <c r="F6" s="26" t="str">
+        <f>TEXT(D6,"mmmm")</f>
+        <v>January</v>
+      </c>
+      <c r="G6" s="27">
+        <f>EOMONTH(D6,0)</f>
+        <v>46053</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>22</v>
       </c>
@@ -3546,8 +3868,24 @@
       <c r="C7" s="2">
         <v>36</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="D7" s="27">
+        <f t="shared" ref="D7:D10" si="0">EDATE(B7,C7)</f>
+        <v>46099</v>
+      </c>
+      <c r="E7" s="26">
+        <f t="shared" ref="E7:E10" si="1">YEAR(D7)</f>
+        <v>2026</v>
+      </c>
+      <c r="F7" s="26" t="str">
+        <f t="shared" ref="F7:F10" si="2">TEXT(D7,"mmmm")</f>
+        <v>March</v>
+      </c>
+      <c r="G7" s="27">
+        <f t="shared" ref="G7:G10" si="3">EOMONTH(D7,0)</f>
+        <v>46112</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -3557,8 +3895,24 @@
       <c r="C8" s="2">
         <v>18</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="D8" s="27">
+        <f t="shared" si="0"/>
+        <v>46381</v>
+      </c>
+      <c r="E8" s="26">
+        <f t="shared" si="1"/>
+        <v>2026</v>
+      </c>
+      <c r="F8" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v>December</v>
+      </c>
+      <c r="G8" s="27">
+        <f t="shared" si="3"/>
+        <v>46387</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>24</v>
       </c>
@@ -3568,8 +3922,24 @@
       <c r="C9" s="2">
         <v>48</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="D9" s="27">
+        <f t="shared" si="0"/>
+        <v>46061</v>
+      </c>
+      <c r="E9" s="26">
+        <f t="shared" si="1"/>
+        <v>2026</v>
+      </c>
+      <c r="F9" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v>February</v>
+      </c>
+      <c r="G9" s="27">
+        <f t="shared" si="3"/>
+        <v>46081</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>30</v>
       </c>
@@ -3579,26 +3949,42 @@
       <c r="C10" s="2">
         <v>12</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" ht="19" x14ac:dyDescent="0.2">
+      <c r="D10" s="27">
+        <f t="shared" si="0"/>
+        <v>45975</v>
+      </c>
+      <c r="E10" s="26">
+        <f t="shared" si="1"/>
+        <v>2025</v>
+      </c>
+      <c r="F10" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v>November</v>
+      </c>
+      <c r="G10" s="27">
+        <f t="shared" si="3"/>
+        <v>45991</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="19" x14ac:dyDescent="0.2">
       <c r="A12" s="14" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="15"/>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" s="15" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="15" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" s="15" t="s">
         <v>162</v>
       </c>
@@ -3615,23 +4001,23 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{475288AA-CC7F-4C0F-AE9A-27205926F7C7}">
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="8" max="8" width="11.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="31" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" ht="31" x14ac:dyDescent="0.2">
       <c r="A1" s="13" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="24" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" ht="24" x14ac:dyDescent="0.2">
       <c r="A3" s="12" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="32" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" ht="48" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>165</v>
       </c>
@@ -3641,8 +4027,20 @@
       <c r="C5" s="3" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="D5" s="32" t="s">
+        <v>206</v>
+      </c>
+      <c r="E5" s="32" t="s">
+        <v>241</v>
+      </c>
+      <c r="F5" s="32" t="s">
+        <v>242</v>
+      </c>
+      <c r="G5" s="32" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>168</v>
       </c>
@@ -3652,8 +4050,24 @@
       <c r="C6" s="2">
         <v>15</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="D6" s="27">
+        <f>B6+C6</f>
+        <v>46228</v>
+      </c>
+      <c r="E6" s="26" t="str">
+        <f>TEXT(D6,"dddd")</f>
+        <v>Saturday</v>
+      </c>
+      <c r="F6" s="26" t="str">
+        <f>TEXT(D6,"mmmm")</f>
+        <v>July</v>
+      </c>
+      <c r="G6" s="27">
+        <f>EOMONTH(D6,0)</f>
+        <v>46234</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>169</v>
       </c>
@@ -3663,8 +4077,24 @@
       <c r="C7" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="D7" s="27">
+        <f t="shared" ref="D7:D10" si="0">B7+C7</f>
+        <v>46245</v>
+      </c>
+      <c r="E7" s="26" t="str">
+        <f t="shared" ref="E7:E10" si="1">TEXT(D7,"dddd")</f>
+        <v>Tuesday</v>
+      </c>
+      <c r="F7" s="26" t="str">
+        <f t="shared" ref="F7:F10" si="2">TEXT(D7,"mmmm")</f>
+        <v>August</v>
+      </c>
+      <c r="G7" s="27">
+        <f t="shared" ref="G7:G10" si="3">EOMONTH(D7,0)</f>
+        <v>46265</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>170</v>
       </c>
@@ -3674,8 +4104,24 @@
       <c r="C8" s="2">
         <v>45</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="D8" s="27">
+        <f t="shared" si="0"/>
+        <v>46263</v>
+      </c>
+      <c r="E8" s="26" t="str">
+        <f t="shared" si="1"/>
+        <v>Saturday</v>
+      </c>
+      <c r="F8" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v>August</v>
+      </c>
+      <c r="G8" s="27">
+        <f t="shared" si="3"/>
+        <v>46265</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>171</v>
       </c>
@@ -3685,8 +4131,24 @@
       <c r="C9" s="2">
         <v>60</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="D9" s="27">
+        <f t="shared" si="0"/>
+        <v>46283</v>
+      </c>
+      <c r="E9" s="26" t="str">
+        <f t="shared" si="1"/>
+        <v>Friday</v>
+      </c>
+      <c r="F9" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v>September</v>
+      </c>
+      <c r="G9" s="27">
+        <f t="shared" si="3"/>
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>172</v>
       </c>
@@ -3696,26 +4158,42 @@
       <c r="C10" s="2">
         <v>90</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" ht="19" x14ac:dyDescent="0.2">
+      <c r="D10" s="27">
+        <f t="shared" si="0"/>
+        <v>46318</v>
+      </c>
+      <c r="E10" s="26" t="str">
+        <f t="shared" si="1"/>
+        <v>Friday</v>
+      </c>
+      <c r="F10" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v>October</v>
+      </c>
+      <c r="G10" s="27">
+        <f t="shared" si="3"/>
+        <v>46326</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="19" x14ac:dyDescent="0.2">
       <c r="A12" s="14" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="15"/>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" s="15" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="15" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" s="15" t="s">
         <v>175</v>
       </c>
@@ -3735,91 +4213,209 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCF54E17-3538-4364-B945-A76B3F1DB769}">
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.1640625" customWidth="1"/>
-    <col min="7" max="7" width="24.33203125" customWidth="1"/>
+    <col min="3" max="3" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="31" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" ht="31" x14ac:dyDescent="0.2">
       <c r="A1" s="13" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="24" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" ht="24" x14ac:dyDescent="0.2">
       <c r="A3" s="12" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>178</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+      <c r="C5" s="29" t="s">
+        <v>244</v>
+      </c>
+      <c r="D5" s="29" t="s">
+        <v>245</v>
+      </c>
+      <c r="E5" s="29" t="s">
+        <v>246</v>
+      </c>
+      <c r="F5" s="29" t="s">
+        <v>247</v>
+      </c>
+      <c r="G5" s="29" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="23" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>180</v>
       </c>
       <c r="B6" s="7">
         <v>46249</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="C6" s="34">
+        <f>WEEKDAY(B6,2)</f>
+        <v>6</v>
+      </c>
+      <c r="D6" s="34" t="str">
+        <f>TEXT(B6,"mmmm")</f>
+        <v>August</v>
+      </c>
+      <c r="E6" s="34">
+        <f>WEEKNUM(B6)</f>
+        <v>33</v>
+      </c>
+      <c r="F6" s="36">
+        <f ca="1">B6-TODAY()</f>
+        <v>-48</v>
+      </c>
+      <c r="G6" s="35">
+        <f>EOMONTH(B6,0)</f>
+        <v>46265</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>181</v>
       </c>
       <c r="B7" s="7">
         <v>46262</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="C7" s="34">
+        <f t="shared" ref="C7:C10" si="0">WEEKDAY(B7,2)</f>
+        <v>5</v>
+      </c>
+      <c r="D7" s="34" t="str">
+        <f t="shared" ref="D7:D10" si="1">TEXT(B7,"mmmm")</f>
+        <v>August</v>
+      </c>
+      <c r="E7" s="34">
+        <f t="shared" ref="E7:E10" si="2">WEEKNUM(B7)</f>
+        <v>35</v>
+      </c>
+      <c r="F7" s="36">
+        <f t="shared" ref="F7:F10" ca="1" si="3">B7-TODAY()</f>
+        <v>-35</v>
+      </c>
+      <c r="G7" s="35">
+        <f t="shared" ref="G7:G10" si="4">EOMONTH(B7,0)</f>
+        <v>46265</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>182</v>
       </c>
       <c r="B8" s="7">
         <v>46277</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="C8" s="34">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="D8" s="34" t="str">
+        <f t="shared" si="1"/>
+        <v>September</v>
+      </c>
+      <c r="E8" s="34">
+        <f t="shared" si="2"/>
+        <v>37</v>
+      </c>
+      <c r="F8" s="36">
+        <f t="shared" ca="1" si="3"/>
+        <v>-20</v>
+      </c>
+      <c r="G8" s="35">
+        <f t="shared" si="4"/>
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="23" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>183</v>
       </c>
       <c r="B9" s="7">
         <v>46320</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="C9" s="34">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="D9" s="34" t="str">
+        <f t="shared" si="1"/>
+        <v>October</v>
+      </c>
+      <c r="E9" s="34">
+        <f t="shared" si="2"/>
+        <v>44</v>
+      </c>
+      <c r="F9" s="36">
+        <f t="shared" ca="1" si="3"/>
+        <v>23</v>
+      </c>
+      <c r="G9" s="35">
+        <f t="shared" si="4"/>
+        <v>46326</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>184</v>
       </c>
       <c r="B10" s="7">
         <v>46344</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" ht="19" x14ac:dyDescent="0.2">
+      <c r="C10" s="34">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="D10" s="34" t="str">
+        <f t="shared" si="1"/>
+        <v>November</v>
+      </c>
+      <c r="E10" s="34">
+        <f t="shared" si="2"/>
+        <v>47</v>
+      </c>
+      <c r="F10" s="36">
+        <f t="shared" ca="1" si="3"/>
+        <v>47</v>
+      </c>
+      <c r="G10" s="35">
+        <f t="shared" si="4"/>
+        <v>46356</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="19" x14ac:dyDescent="0.2">
       <c r="A12" s="14" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="15"/>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" s="15" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="15" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" s="15" t="s">
         <v>187</v>
       </c>

</xml_diff>